<commit_message>
wMKL re-run; consensus and comparisons update
</commit_message>
<xml_diff>
--- a/Resources/Runtimes.xlsx
+++ b/Resources/Runtimes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/as3582_cam_ac_uk/Documents/Desktop/GitHub/MultiOmicsSurvey/Resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\as3582\OneDrive - University of Cambridge\Desktop\GitHub\MultiOmicsSurvey\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="13_ncr:1_{A7AA482A-EA94-4862-B88A-03EEEC75368F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{968C6517-E08A-4952-B9EE-1DCB5BD1D071}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2883A655-894A-4D57-B165-3F901F8C8181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44310" yWindow="1635" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -473,20 +473,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" style="2" customWidth="1"/>
     <col min="3" max="3" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.08984375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="133.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" style="2"/>
+    <col min="4" max="4" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="133.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,7 +512,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -536,7 +536,7 @@
         <v>3.1111111111111112</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -560,7 +560,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -584,7 +584,7 @@
         <v>0.23148148148148148</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -611,7 +611,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -635,7 +635,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -662,7 +662,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -689,7 +689,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -713,7 +713,7 @@
         <v>3.1111111111111112</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -740,7 +740,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
@@ -767,7 +767,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>14</v>
       </c>
@@ -791,7 +791,7 @@
         <v>1.4867480468750001</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
@@ -808,14 +808,14 @@
         <v>1</v>
       </c>
       <c r="F13" s="2">
-        <v>4.5</v>
+        <v>7.04</v>
       </c>
       <c r="G13" s="2">
         <f t="shared" si="0"/>
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+        <v>7.04</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
@@ -839,7 +839,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -866,7 +866,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
@@ -890,7 +890,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -917,7 +917,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -941,7 +941,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>21</v>
       </c>

</xml_diff>